<commit_message>
Added BOM and Gerbers
BOM and Gerbers, ready to be sent to PCB manufacturer
</commit_message>
<xml_diff>
--- a/4_Schematics and Boards Layout/4_7_Production Files/Gerber_PowerBoard/CPL.xlsx
+++ b/4_Schematics and Boards Layout/4_7_Production Files/Gerber_PowerBoard/CPL.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="PowerBoard" localSheetId="0">Feuil1!$A$2:$G$277</definedName>
+    <definedName name="PowerBoard" localSheetId="0">Feuil1!$A$2:$E$277</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <connection id="1" name="PowerBoard" type="6" refreshedVersion="3" background="1" saveData="1">
-    <textPr codePage="932" sourceFile="C:\Users\dell\Desktop\CrowdSupply\RADAR_V6\4_Schematics and Boards Layout\4_6_Schematics\PowerBoard\Gerber_PowerBoard\PowerBoard.mnt" decimal="," thousands=" " space="1" consecutive="1">
+    <textPr codePage="932" sourceFile="C:\Users\dell\Desktop\CrowdSupply\RADAR_V6\4_Schematics and Boards Layout\4_7_Production Files\Gerber_PowerBoard\PowerBoard.mnt" decimal="," thousands=" " space="1" consecutive="1">
       <textFields count="6">
         <textField/>
         <textField/>
@@ -2300,30 +2300,38 @@
     <t>279.40</t>
   </si>
   <si>
-    <t>Designator</t>
-  </si>
-  <si>
-    <t>Mid_X(mm)</t>
-  </si>
-  <si>
-    <t>Mid_Y(mm)</t>
+    <t>DESIGNATOR</t>
+  </si>
+  <si>
+    <t>Mid X (mm)</t>
+  </si>
+  <si>
+    <t>Mid Y (mm)</t>
   </si>
   <si>
     <t>Layer</t>
   </si>
   <si>
+    <t>Top</t>
+  </si>
+  <si>
     <t>Rotation</t>
-  </si>
-  <si>
-    <t>Top</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2351,8 +2359,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2654,30 +2663,28 @@
   <dimension ref="A1:E277"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
         <v>754</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>755</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>756</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>757</v>
       </c>
-      <c r="E1" t="s">
-        <v>758</v>
+      <c r="E1" s="1" t="s">
+        <v>759</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2691,7 +2698,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E2">
         <v>90</v>
@@ -2708,7 +2715,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2725,7 +2732,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -2742,7 +2749,7 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E5">
         <v>90</v>
@@ -2759,7 +2766,7 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E6">
         <v>90</v>
@@ -2776,7 +2783,7 @@
         <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E7">
         <v>90</v>
@@ -2793,7 +2800,7 @@
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -2810,7 +2817,7 @@
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -2827,7 +2834,7 @@
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E10">
         <v>90</v>
@@ -2844,7 +2851,7 @@
         <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E11">
         <v>90</v>
@@ -2861,7 +2868,7 @@
         <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -2878,7 +2885,7 @@
         <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E13">
         <v>90</v>
@@ -2895,7 +2902,7 @@
         <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -2912,7 +2919,7 @@
         <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2929,7 +2936,7 @@
         <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E16">
         <v>90</v>
@@ -2946,7 +2953,7 @@
         <v>43</v>
       </c>
       <c r="D17" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E17">
         <v>90</v>
@@ -2963,7 +2970,7 @@
         <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -2980,7 +2987,7 @@
         <v>48</v>
       </c>
       <c r="D19" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E19">
         <v>90</v>
@@ -2997,7 +3004,7 @@
         <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -3014,7 +3021,7 @@
         <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -3031,7 +3038,7 @@
         <v>56</v>
       </c>
       <c r="D22" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E22">
         <v>90</v>
@@ -3048,7 +3055,7 @@
         <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E23">
         <v>90</v>
@@ -3065,7 +3072,7 @@
         <v>60</v>
       </c>
       <c r="D24" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -3082,7 +3089,7 @@
         <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -3099,7 +3106,7 @@
         <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E26">
         <v>90</v>
@@ -3116,7 +3123,7 @@
         <v>69</v>
       </c>
       <c r="D27" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -3133,7 +3140,7 @@
         <v>72</v>
       </c>
       <c r="D28" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E28">
         <v>180</v>
@@ -3150,7 +3157,7 @@
         <v>63</v>
       </c>
       <c r="D29" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E29">
         <v>180</v>
@@ -3167,7 +3174,7 @@
         <v>77</v>
       </c>
       <c r="D30" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -3184,7 +3191,7 @@
         <v>80</v>
       </c>
       <c r="D31" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E31">
         <v>90</v>
@@ -3201,7 +3208,7 @@
         <v>83</v>
       </c>
       <c r="D32" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -3218,7 +3225,7 @@
         <v>85</v>
       </c>
       <c r="D33" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -3235,7 +3242,7 @@
         <v>88</v>
       </c>
       <c r="D34" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E34">
         <v>90</v>
@@ -3252,7 +3259,7 @@
         <v>88</v>
       </c>
       <c r="D35" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E35">
         <v>90</v>
@@ -3269,7 +3276,7 @@
         <v>92</v>
       </c>
       <c r="D36" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -3286,7 +3293,7 @@
         <v>95</v>
       </c>
       <c r="D37" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E37">
         <v>90</v>
@@ -3303,7 +3310,7 @@
         <v>98</v>
       </c>
       <c r="D38" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -3320,7 +3327,7 @@
         <v>100</v>
       </c>
       <c r="D39" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -3337,7 +3344,7 @@
         <v>103</v>
       </c>
       <c r="D40" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E40">
         <v>90</v>
@@ -3354,7 +3361,7 @@
         <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E41">
         <v>90</v>
@@ -3371,7 +3378,7 @@
         <v>107</v>
       </c>
       <c r="D42" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -3388,7 +3395,7 @@
         <v>110</v>
       </c>
       <c r="D43" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E43">
         <v>90</v>
@@ -3405,7 +3412,7 @@
         <v>113</v>
       </c>
       <c r="D44" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -3422,7 +3429,7 @@
         <v>115</v>
       </c>
       <c r="D45" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E45">
         <v>0</v>
@@ -3439,7 +3446,7 @@
         <v>118</v>
       </c>
       <c r="D46" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E46">
         <v>90</v>
@@ -3456,7 +3463,7 @@
         <v>118</v>
       </c>
       <c r="D47" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E47">
         <v>90</v>
@@ -3473,7 +3480,7 @@
         <v>123</v>
       </c>
       <c r="D48" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3490,7 +3497,7 @@
         <v>126</v>
       </c>
       <c r="D49" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -3507,7 +3514,7 @@
         <v>128</v>
       </c>
       <c r="D50" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -3524,7 +3531,7 @@
         <v>131</v>
       </c>
       <c r="D51" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E51">
         <v>90</v>
@@ -3541,7 +3548,7 @@
         <v>131</v>
       </c>
       <c r="D52" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E52">
         <v>90</v>
@@ -3558,7 +3565,7 @@
         <v>136</v>
       </c>
       <c r="D53" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -3575,7 +3582,7 @@
         <v>139</v>
       </c>
       <c r="D54" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E54">
         <v>90</v>
@@ -3592,7 +3599,7 @@
         <v>142</v>
       </c>
       <c r="D55" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E55">
         <v>90</v>
@@ -3609,7 +3616,7 @@
         <v>145</v>
       </c>
       <c r="D56" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -3626,7 +3633,7 @@
         <v>147</v>
       </c>
       <c r="D57" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -3643,7 +3650,7 @@
         <v>150</v>
       </c>
       <c r="D58" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E58">
         <v>90</v>
@@ -3660,7 +3667,7 @@
         <v>150</v>
       </c>
       <c r="D59" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E59">
         <v>90</v>
@@ -3677,7 +3684,7 @@
         <v>153</v>
       </c>
       <c r="D60" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3694,7 +3701,7 @@
         <v>156</v>
       </c>
       <c r="D61" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E61">
         <v>90</v>
@@ -3711,7 +3718,7 @@
         <v>159</v>
       </c>
       <c r="D62" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3728,7 +3735,7 @@
         <v>161</v>
       </c>
       <c r="D63" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3745,7 +3752,7 @@
         <v>164</v>
       </c>
       <c r="D64" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E64">
         <v>90</v>
@@ -3762,7 +3769,7 @@
         <v>164</v>
       </c>
       <c r="D65" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E65">
         <v>90</v>
@@ -3779,7 +3786,7 @@
         <v>168</v>
       </c>
       <c r="D66" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3796,7 +3803,7 @@
         <v>171</v>
       </c>
       <c r="D67" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E67">
         <v>90</v>
@@ -3813,7 +3820,7 @@
         <v>174</v>
       </c>
       <c r="D68" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3830,7 +3837,7 @@
         <v>176</v>
       </c>
       <c r="D69" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -3847,7 +3854,7 @@
         <v>179</v>
       </c>
       <c r="D70" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E70">
         <v>90</v>
@@ -3864,7 +3871,7 @@
         <v>179</v>
       </c>
       <c r="D71" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E71">
         <v>90</v>
@@ -3881,7 +3888,7 @@
         <v>184</v>
       </c>
       <c r="D72" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E72">
         <v>90</v>
@@ -3898,7 +3905,7 @@
         <v>187</v>
       </c>
       <c r="D73" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E73">
         <v>0</v>
@@ -3915,7 +3922,7 @@
         <v>189</v>
       </c>
       <c r="D74" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -3932,7 +3939,7 @@
         <v>192</v>
       </c>
       <c r="D75" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E75">
         <v>90</v>
@@ -3949,7 +3956,7 @@
         <v>192</v>
       </c>
       <c r="D76" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E76">
         <v>90</v>
@@ -3966,7 +3973,7 @@
         <v>197</v>
       </c>
       <c r="D77" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E77">
         <v>90</v>
@@ -3983,7 +3990,7 @@
         <v>200</v>
       </c>
       <c r="D78" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E78">
         <v>90</v>
@@ -4000,7 +4007,7 @@
         <v>203</v>
       </c>
       <c r="D79" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -4017,7 +4024,7 @@
         <v>205</v>
       </c>
       <c r="D80" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -4034,7 +4041,7 @@
         <v>208</v>
       </c>
       <c r="D81" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E81">
         <v>90</v>
@@ -4051,7 +4058,7 @@
         <v>208</v>
       </c>
       <c r="D82" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E82">
         <v>90</v>
@@ -4068,7 +4075,7 @@
         <v>213</v>
       </c>
       <c r="D83" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E83">
         <v>0</v>
@@ -4085,7 +4092,7 @@
         <v>216</v>
       </c>
       <c r="D84" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E84">
         <v>90</v>
@@ -4102,7 +4109,7 @@
         <v>219</v>
       </c>
       <c r="D85" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E85">
         <v>0</v>
@@ -4119,7 +4126,7 @@
         <v>221</v>
       </c>
       <c r="D86" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -4136,7 +4143,7 @@
         <v>224</v>
       </c>
       <c r="D87" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E87">
         <v>90</v>
@@ -4153,7 +4160,7 @@
         <v>224</v>
       </c>
       <c r="D88" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E88">
         <v>90</v>
@@ -4170,7 +4177,7 @@
         <v>228</v>
       </c>
       <c r="D89" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E89">
         <v>0</v>
@@ -4187,7 +4194,7 @@
         <v>231</v>
       </c>
       <c r="D90" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E90">
         <v>90</v>
@@ -4204,7 +4211,7 @@
         <v>234</v>
       </c>
       <c r="D91" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E91">
         <v>0</v>
@@ -4221,7 +4228,7 @@
         <v>236</v>
       </c>
       <c r="D92" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E92">
         <v>0</v>
@@ -4238,7 +4245,7 @@
         <v>239</v>
       </c>
       <c r="D93" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E93">
         <v>90</v>
@@ -4255,7 +4262,7 @@
         <v>239</v>
       </c>
       <c r="D94" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E94">
         <v>90</v>
@@ -4272,7 +4279,7 @@
         <v>244</v>
       </c>
       <c r="D95" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E95">
         <v>90</v>
@@ -4289,7 +4296,7 @@
         <v>244</v>
       </c>
       <c r="D96" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E96">
         <v>90</v>
@@ -4306,7 +4313,7 @@
         <v>249</v>
       </c>
       <c r="D97" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E97">
         <v>180</v>
@@ -4323,7 +4330,7 @@
         <v>252</v>
       </c>
       <c r="D98" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E98">
         <v>0</v>
@@ -4340,7 +4347,7 @@
         <v>255</v>
       </c>
       <c r="D99" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E99">
         <v>180</v>
@@ -4357,7 +4364,7 @@
         <v>258</v>
       </c>
       <c r="D100" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E100">
         <v>90</v>
@@ -4374,7 +4381,7 @@
         <v>261</v>
       </c>
       <c r="D101" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E101">
         <v>180</v>
@@ -4391,7 +4398,7 @@
         <v>264</v>
       </c>
       <c r="D102" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E102">
         <v>90</v>
@@ -4408,7 +4415,7 @@
         <v>267</v>
       </c>
       <c r="D103" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E103">
         <v>0</v>
@@ -4425,7 +4432,7 @@
         <v>270</v>
       </c>
       <c r="D104" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E104">
         <v>90</v>
@@ -4442,7 +4449,7 @@
         <v>273</v>
       </c>
       <c r="D105" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E105">
         <v>270</v>
@@ -4459,7 +4466,7 @@
         <v>276</v>
       </c>
       <c r="D106" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E106">
         <v>90</v>
@@ -4476,7 +4483,7 @@
         <v>279</v>
       </c>
       <c r="D107" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -4493,7 +4500,7 @@
         <v>282</v>
       </c>
       <c r="D108" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E108">
         <v>180</v>
@@ -4510,7 +4517,7 @@
         <v>136</v>
       </c>
       <c r="D109" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E109">
         <v>180</v>
@@ -4527,7 +4534,7 @@
         <v>287</v>
       </c>
       <c r="D110" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E110">
         <v>90</v>
@@ -4544,7 +4551,7 @@
         <v>290</v>
       </c>
       <c r="D111" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E111">
         <v>0</v>
@@ -4561,7 +4568,7 @@
         <v>292</v>
       </c>
       <c r="D112" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E112">
         <v>0</v>
@@ -4578,7 +4585,7 @@
         <v>295</v>
       </c>
       <c r="D113" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E113">
         <v>90</v>
@@ -4595,7 +4602,7 @@
         <v>295</v>
       </c>
       <c r="D114" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E114">
         <v>90</v>
@@ -4612,7 +4619,7 @@
         <v>300</v>
       </c>
       <c r="D115" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E115">
         <v>0</v>
@@ -4629,7 +4636,7 @@
         <v>303</v>
       </c>
       <c r="D116" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E116">
         <v>90</v>
@@ -4646,7 +4653,7 @@
         <v>306</v>
       </c>
       <c r="D117" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E117">
         <v>0</v>
@@ -4663,7 +4670,7 @@
         <v>309</v>
       </c>
       <c r="D118" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E118">
         <v>180</v>
@@ -4680,7 +4687,7 @@
         <v>312</v>
       </c>
       <c r="D119" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E119">
         <v>180</v>
@@ -4697,7 +4704,7 @@
         <v>315</v>
       </c>
       <c r="D120" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E120">
         <v>90</v>
@@ -4714,7 +4721,7 @@
         <v>318</v>
       </c>
       <c r="D121" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E121">
         <v>0</v>
@@ -4731,7 +4738,7 @@
         <v>321</v>
       </c>
       <c r="D122" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E122">
         <v>0</v>
@@ -4748,7 +4755,7 @@
         <v>324</v>
       </c>
       <c r="D123" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E123">
         <v>90</v>
@@ -4765,7 +4772,7 @@
         <v>324</v>
       </c>
       <c r="D124" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E124">
         <v>90</v>
@@ -4782,7 +4789,7 @@
         <v>329</v>
       </c>
       <c r="D125" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E125">
         <v>0</v>
@@ -4799,7 +4806,7 @@
         <v>332</v>
       </c>
       <c r="D126" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E126">
         <v>90</v>
@@ -4816,7 +4823,7 @@
         <v>335</v>
       </c>
       <c r="D127" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E127">
         <v>0</v>
@@ -4833,7 +4840,7 @@
         <v>338</v>
       </c>
       <c r="D128" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E128">
         <v>180</v>
@@ -4850,7 +4857,7 @@
         <v>329</v>
       </c>
       <c r="D129" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E129">
         <v>180</v>
@@ -4867,7 +4874,7 @@
         <v>343</v>
       </c>
       <c r="D130" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E130">
         <v>90</v>
@@ -4884,7 +4891,7 @@
         <v>346</v>
       </c>
       <c r="D131" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E131">
         <v>0</v>
@@ -4901,7 +4908,7 @@
         <v>348</v>
       </c>
       <c r="D132" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E132">
         <v>0</v>
@@ -4918,7 +4925,7 @@
         <v>324</v>
       </c>
       <c r="D133" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E133">
         <v>90</v>
@@ -4935,7 +4942,7 @@
         <v>324</v>
       </c>
       <c r="D134" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E134">
         <v>90</v>
@@ -4952,7 +4959,7 @@
         <v>355</v>
       </c>
       <c r="D135" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E135">
         <v>0</v>
@@ -4969,7 +4976,7 @@
         <v>332</v>
       </c>
       <c r="D136" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E136">
         <v>90</v>
@@ -4986,7 +4993,7 @@
         <v>360</v>
       </c>
       <c r="D137" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E137">
         <v>0</v>
@@ -5003,7 +5010,7 @@
         <v>363</v>
       </c>
       <c r="D138" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E138">
         <v>180</v>
@@ -5020,7 +5027,7 @@
         <v>366</v>
       </c>
       <c r="D139" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E139">
         <v>180</v>
@@ -5037,7 +5044,7 @@
         <v>369</v>
       </c>
       <c r="D140" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E140">
         <v>0</v>
@@ -5054,7 +5061,7 @@
         <v>372</v>
       </c>
       <c r="D141" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E141">
         <v>90</v>
@@ -5071,7 +5078,7 @@
         <v>375</v>
       </c>
       <c r="D142" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E142">
         <v>0</v>
@@ -5088,7 +5095,7 @@
         <v>378</v>
       </c>
       <c r="D143" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E143">
         <v>180</v>
@@ -5105,7 +5112,7 @@
         <v>381</v>
       </c>
       <c r="D144" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E144">
         <v>180</v>
@@ -5122,7 +5129,7 @@
         <v>384</v>
       </c>
       <c r="D145" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E145">
         <v>90</v>
@@ -5139,7 +5146,7 @@
         <v>387</v>
       </c>
       <c r="D146" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E146">
         <v>0</v>
@@ -5156,7 +5163,7 @@
         <v>389</v>
       </c>
       <c r="D147" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E147">
         <v>0</v>
@@ -5173,7 +5180,7 @@
         <v>392</v>
       </c>
       <c r="D148" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E148">
         <v>90</v>
@@ -5190,7 +5197,7 @@
         <v>392</v>
       </c>
       <c r="D149" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E149">
         <v>90</v>
@@ -5207,7 +5214,7 @@
         <v>397</v>
       </c>
       <c r="D150" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E150">
         <v>270</v>
@@ -5224,7 +5231,7 @@
         <v>400</v>
       </c>
       <c r="D151" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E151">
         <v>90</v>
@@ -5241,7 +5248,7 @@
         <v>403</v>
       </c>
       <c r="D152" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E152">
         <v>90</v>
@@ -5258,7 +5265,7 @@
         <v>400</v>
       </c>
       <c r="D153" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E153">
         <v>90</v>
@@ -5275,7 +5282,7 @@
         <v>408</v>
       </c>
       <c r="D154" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E154">
         <v>0</v>
@@ -5292,7 +5299,7 @@
         <v>411</v>
       </c>
       <c r="D155" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E155">
         <v>90</v>
@@ -5309,7 +5316,7 @@
         <v>414</v>
       </c>
       <c r="D156" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E156">
         <v>0</v>
@@ -5326,7 +5333,7 @@
         <v>417</v>
       </c>
       <c r="D157" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E157">
         <v>0</v>
@@ -5343,7 +5350,7 @@
         <v>420</v>
       </c>
       <c r="D158" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E158">
         <v>90</v>
@@ -5360,7 +5367,7 @@
         <v>420</v>
       </c>
       <c r="D159" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E159">
         <v>90</v>
@@ -5377,7 +5384,7 @@
         <v>425</v>
       </c>
       <c r="D160" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E160">
         <v>270</v>
@@ -5394,7 +5401,7 @@
         <v>428</v>
       </c>
       <c r="D161" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E161">
         <v>90</v>
@@ -5411,7 +5418,7 @@
         <v>431</v>
       </c>
       <c r="D162" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E162">
         <v>90</v>
@@ -5428,7 +5435,7 @@
         <v>434</v>
       </c>
       <c r="D163" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E163">
         <v>90</v>
@@ -5445,7 +5452,7 @@
         <v>437</v>
       </c>
       <c r="D164" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E164">
         <v>0</v>
@@ -5462,7 +5469,7 @@
         <v>440</v>
       </c>
       <c r="D165" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E165">
         <v>90</v>
@@ -5479,7 +5486,7 @@
         <v>443</v>
       </c>
       <c r="D166" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E166">
         <v>270</v>
@@ -5496,7 +5503,7 @@
         <v>440</v>
       </c>
       <c r="D167" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E167">
         <v>90</v>
@@ -5513,7 +5520,7 @@
         <v>448</v>
       </c>
       <c r="D168" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E168">
         <v>270</v>
@@ -5530,7 +5537,7 @@
         <v>451</v>
       </c>
       <c r="D169" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E169">
         <v>90</v>
@@ -5547,7 +5554,7 @@
         <v>454</v>
       </c>
       <c r="D170" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E170">
         <v>270</v>
@@ -5564,7 +5571,7 @@
         <v>457</v>
       </c>
       <c r="D171" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E171">
         <v>90</v>
@@ -5581,7 +5588,7 @@
         <v>460</v>
       </c>
       <c r="D172" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E172">
         <v>270</v>
@@ -5598,7 +5605,7 @@
         <v>463</v>
       </c>
       <c r="D173" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E173">
         <v>0</v>
@@ -5615,7 +5622,7 @@
         <v>463</v>
       </c>
       <c r="D174" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E174">
         <v>0</v>
@@ -5632,7 +5639,7 @@
         <v>468</v>
       </c>
       <c r="D175" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E175">
         <v>90</v>
@@ -5649,7 +5656,7 @@
         <v>471</v>
       </c>
       <c r="D176" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E176">
         <v>270</v>
@@ -5666,7 +5673,7 @@
         <v>474</v>
       </c>
       <c r="D177" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E177">
         <v>90</v>
@@ -5683,7 +5690,7 @@
         <v>477</v>
       </c>
       <c r="D178" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E178">
         <v>270</v>
@@ -5700,7 +5707,7 @@
         <v>480</v>
       </c>
       <c r="D179" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E179">
         <v>90</v>
@@ -5717,7 +5724,7 @@
         <v>483</v>
       </c>
       <c r="D180" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E180">
         <v>270</v>
@@ -5734,7 +5741,7 @@
         <v>486</v>
       </c>
       <c r="D181" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E181">
         <v>90</v>
@@ -5751,7 +5758,7 @@
         <v>486</v>
       </c>
       <c r="D182" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E182">
         <v>270</v>
@@ -5768,7 +5775,7 @@
         <v>491</v>
       </c>
       <c r="D183" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E183">
         <v>90</v>
@@ -5785,7 +5792,7 @@
         <v>491</v>
       </c>
       <c r="D184" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E184">
         <v>270</v>
@@ -5802,7 +5809,7 @@
         <v>496</v>
       </c>
       <c r="D185" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E185">
         <v>90</v>
@@ -5819,7 +5826,7 @@
         <v>499</v>
       </c>
       <c r="D186" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E186">
         <v>270</v>
@@ -5836,7 +5843,7 @@
         <v>502</v>
       </c>
       <c r="D187" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E187">
         <v>90</v>
@@ -5853,7 +5860,7 @@
         <v>505</v>
       </c>
       <c r="D188" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E188">
         <v>270</v>
@@ -5870,7 +5877,7 @@
         <v>508</v>
       </c>
       <c r="D189" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E189">
         <v>90</v>
@@ -5887,7 +5894,7 @@
         <v>511</v>
       </c>
       <c r="D190" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E190">
         <v>270</v>
@@ -5904,7 +5911,7 @@
         <v>514</v>
       </c>
       <c r="D191" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E191">
         <v>90</v>
@@ -5921,7 +5928,7 @@
         <v>517</v>
       </c>
       <c r="D192" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E192">
         <v>270</v>
@@ -5938,7 +5945,7 @@
         <v>520</v>
       </c>
       <c r="D193" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E193">
         <v>90</v>
@@ -5955,7 +5962,7 @@
         <v>523</v>
       </c>
       <c r="D194" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E194">
         <v>270</v>
@@ -5972,7 +5979,7 @@
         <v>224</v>
       </c>
       <c r="D195" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E195">
         <v>90</v>
@@ -5989,7 +5996,7 @@
         <v>528</v>
       </c>
       <c r="D196" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E196">
         <v>270</v>
@@ -6006,7 +6013,7 @@
         <v>530</v>
       </c>
       <c r="D197" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E197">
         <v>90</v>
@@ -6023,7 +6030,7 @@
         <v>533</v>
       </c>
       <c r="D198" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E198">
         <v>270</v>
@@ -6040,7 +6047,7 @@
         <v>536</v>
       </c>
       <c r="D199" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E199">
         <v>0</v>
@@ -6057,7 +6064,7 @@
         <v>539</v>
       </c>
       <c r="D200" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E200">
         <v>0</v>
@@ -6074,7 +6081,7 @@
         <v>542</v>
       </c>
       <c r="D201" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E201">
         <v>90</v>
@@ -6091,7 +6098,7 @@
         <v>542</v>
       </c>
       <c r="D202" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E202">
         <v>270</v>
@@ -6108,7 +6115,7 @@
         <v>546</v>
       </c>
       <c r="D203" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E203">
         <v>0</v>
@@ -6125,7 +6132,7 @@
         <v>546</v>
       </c>
       <c r="D204" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E204">
         <v>0</v>
@@ -6142,7 +6149,7 @@
         <v>551</v>
       </c>
       <c r="D205" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E205">
         <v>90</v>
@@ -6159,7 +6166,7 @@
         <v>554</v>
       </c>
       <c r="D206" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E206">
         <v>270</v>
@@ -6176,7 +6183,7 @@
         <v>557</v>
       </c>
       <c r="D207" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E207">
         <v>0</v>
@@ -6193,7 +6200,7 @@
         <v>557</v>
       </c>
       <c r="D208" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E208">
         <v>0</v>
@@ -6210,7 +6217,7 @@
         <v>562</v>
       </c>
       <c r="D209" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E209">
         <v>90</v>
@@ -6227,7 +6234,7 @@
         <v>562</v>
       </c>
       <c r="D210" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E210">
         <v>270</v>
@@ -6244,7 +6251,7 @@
         <v>567</v>
       </c>
       <c r="D211" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E211">
         <v>0</v>
@@ -6261,7 +6268,7 @@
         <v>567</v>
       </c>
       <c r="D212" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E212">
         <v>0</v>
@@ -6278,7 +6285,7 @@
         <v>571</v>
       </c>
       <c r="D213" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E213">
         <v>0</v>
@@ -6295,7 +6302,7 @@
         <v>571</v>
       </c>
       <c r="D214" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E214">
         <v>0</v>
@@ -6312,7 +6319,7 @@
         <v>576</v>
       </c>
       <c r="D215" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E215">
         <v>90</v>
@@ -6329,7 +6336,7 @@
         <v>579</v>
       </c>
       <c r="D216" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E216">
         <v>270</v>
@@ -6346,7 +6353,7 @@
         <v>400</v>
       </c>
       <c r="D217" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E217">
         <v>270</v>
@@ -6363,7 +6370,7 @@
         <v>584</v>
       </c>
       <c r="D218" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E218">
         <v>0</v>
@@ -6380,7 +6387,7 @@
         <v>420</v>
       </c>
       <c r="D219" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E219">
         <v>90</v>
@@ -6397,7 +6404,7 @@
         <v>420</v>
       </c>
       <c r="D220" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E220">
         <v>270</v>
@@ -6414,7 +6421,7 @@
         <v>591</v>
       </c>
       <c r="D221" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E221">
         <v>270</v>
@@ -6431,7 +6438,7 @@
         <v>594</v>
       </c>
       <c r="D222" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E222">
         <v>270</v>
@@ -6448,7 +6455,7 @@
         <v>597</v>
       </c>
       <c r="D223" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E223">
         <v>270</v>
@@ -6465,7 +6472,7 @@
         <v>600</v>
       </c>
       <c r="D224" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E224">
         <v>270</v>
@@ -6482,7 +6489,7 @@
         <v>2</v>
       </c>
       <c r="D225" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E225">
         <v>270</v>
@@ -6499,7 +6506,7 @@
         <v>605</v>
       </c>
       <c r="D226" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E226">
         <v>270</v>
@@ -6516,7 +6523,7 @@
         <v>608</v>
       </c>
       <c r="D227" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E227">
         <v>270</v>
@@ -6533,7 +6540,7 @@
         <v>611</v>
       </c>
       <c r="D228" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E228">
         <v>270</v>
@@ -6550,7 +6557,7 @@
         <v>614</v>
       </c>
       <c r="D229" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E229">
         <v>270</v>
@@ -6567,7 +6574,7 @@
         <v>617</v>
       </c>
       <c r="D230" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E230">
         <v>270</v>
@@ -6584,7 +6591,7 @@
         <v>620</v>
       </c>
       <c r="D231" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E231">
         <v>270</v>
@@ -6601,7 +6608,7 @@
         <v>623</v>
       </c>
       <c r="D232" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E232">
         <v>270</v>
@@ -6618,7 +6625,7 @@
         <v>626</v>
       </c>
       <c r="D233" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E233">
         <v>270</v>
@@ -6635,7 +6642,7 @@
         <v>629</v>
       </c>
       <c r="D234" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E234">
         <v>270</v>
@@ -6652,7 +6659,7 @@
         <v>632</v>
       </c>
       <c r="D235" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E235">
         <v>270</v>
@@ -6669,7 +6676,7 @@
         <v>635</v>
       </c>
       <c r="D236" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E236">
         <v>270</v>
@@ -6686,7 +6693,7 @@
         <v>638</v>
       </c>
       <c r="D237" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E237">
         <v>270</v>
@@ -6703,7 +6710,7 @@
         <v>641</v>
       </c>
       <c r="D238" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E238">
         <v>270</v>
@@ -6720,7 +6727,7 @@
         <v>644</v>
       </c>
       <c r="D239" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E239">
         <v>270</v>
@@ -6737,7 +6744,7 @@
         <v>646</v>
       </c>
       <c r="D240" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E240">
         <v>270</v>
@@ -6754,7 +6761,7 @@
         <v>649</v>
       </c>
       <c r="D241" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E241">
         <v>270</v>
@@ -6771,7 +6778,7 @@
         <v>652</v>
       </c>
       <c r="D242" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E242">
         <v>270</v>
@@ -6788,7 +6795,7 @@
         <v>655</v>
       </c>
       <c r="D243" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E243">
         <v>270</v>
@@ -6805,7 +6812,7 @@
         <v>658</v>
       </c>
       <c r="D244" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E244">
         <v>0</v>
@@ -6822,7 +6829,7 @@
         <v>661</v>
       </c>
       <c r="D245" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E245">
         <v>0</v>
@@ -6839,7 +6846,7 @@
         <v>661</v>
       </c>
       <c r="D246" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E246">
         <v>0</v>
@@ -6856,7 +6863,7 @@
         <v>666</v>
       </c>
       <c r="D247" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E247">
         <v>0</v>
@@ -6873,7 +6880,7 @@
         <v>669</v>
       </c>
       <c r="D248" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E248">
         <v>180</v>
@@ -6890,7 +6897,7 @@
         <v>672</v>
       </c>
       <c r="D249" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E249">
         <v>0</v>
@@ -6907,7 +6914,7 @@
         <v>477</v>
       </c>
       <c r="D250" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E250">
         <v>0</v>
@@ -6924,7 +6931,7 @@
         <v>677</v>
       </c>
       <c r="D251" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E251">
         <v>0</v>
@@ -6941,7 +6948,7 @@
         <v>680</v>
       </c>
       <c r="D252" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E252">
         <v>0</v>
@@ -6958,7 +6965,7 @@
         <v>683</v>
       </c>
       <c r="D253" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E253">
         <v>0</v>
@@ -6975,7 +6982,7 @@
         <v>686</v>
       </c>
       <c r="D254" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E254">
         <v>0</v>
@@ -6992,7 +6999,7 @@
         <v>505</v>
       </c>
       <c r="D255" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E255">
         <v>0</v>
@@ -7009,7 +7016,7 @@
         <v>691</v>
       </c>
       <c r="D256" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E256">
         <v>0</v>
@@ -7026,7 +7033,7 @@
         <v>694</v>
       </c>
       <c r="D257" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E257">
         <v>0</v>
@@ -7043,7 +7050,7 @@
         <v>697</v>
       </c>
       <c r="D258" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E258">
         <v>0</v>
@@ -7060,7 +7067,7 @@
         <v>700</v>
       </c>
       <c r="D259" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E259">
         <v>0</v>
@@ -7077,7 +7084,7 @@
         <v>703</v>
       </c>
       <c r="D260" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E260">
         <v>0</v>
@@ -7094,7 +7101,7 @@
         <v>706</v>
       </c>
       <c r="D261" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E261">
         <v>270</v>
@@ -7111,7 +7118,7 @@
         <v>709</v>
       </c>
       <c r="D262" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E262">
         <v>270</v>
@@ -7128,7 +7135,7 @@
         <v>712</v>
       </c>
       <c r="D263" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E263">
         <v>270</v>
@@ -7145,7 +7152,7 @@
         <v>715</v>
       </c>
       <c r="D264" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E264">
         <v>90</v>
@@ -7162,7 +7169,7 @@
         <v>718</v>
       </c>
       <c r="D265" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E265">
         <v>0</v>
@@ -7179,7 +7186,7 @@
         <v>721</v>
       </c>
       <c r="D266" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E266">
         <v>180</v>
@@ -7196,7 +7203,7 @@
         <v>724</v>
       </c>
       <c r="D267" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E267">
         <v>0</v>
@@ -7213,7 +7220,7 @@
         <v>727</v>
       </c>
       <c r="D268" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E268">
         <v>180</v>
@@ -7230,7 +7237,7 @@
         <v>730</v>
       </c>
       <c r="D269" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E269">
         <v>0</v>
@@ -7247,7 +7254,7 @@
         <v>733</v>
       </c>
       <c r="D270" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E270">
         <v>180</v>
@@ -7264,7 +7271,7 @@
         <v>736</v>
       </c>
       <c r="D271" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E271">
         <v>0</v>
@@ -7281,7 +7288,7 @@
         <v>739</v>
       </c>
       <c r="D272" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E272">
         <v>180</v>
@@ -7298,7 +7305,7 @@
         <v>742</v>
       </c>
       <c r="D273" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E273">
         <v>180</v>
@@ -7315,7 +7322,7 @@
         <v>745</v>
       </c>
       <c r="D274" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E274">
         <v>0</v>
@@ -7332,7 +7339,7 @@
         <v>748</v>
       </c>
       <c r="D275" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E275">
         <v>180</v>
@@ -7349,7 +7356,7 @@
         <v>730</v>
       </c>
       <c r="D276" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E276">
         <v>0</v>
@@ -7366,7 +7373,7 @@
         <v>753</v>
       </c>
       <c r="D277" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E277">
         <v>180</v>
@@ -7374,6 +7381,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>